<commit_message>
updating after comparison with some original xl files
</commit_message>
<xml_diff>
--- a/AutocallPricer.xlsx
+++ b/AutocallPricer.xlsx
@@ -1,29 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antoine\Source\Repos\CompFinance\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bernardo\dev\repos\CompFinance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F814CD88-FA55-4FA1-BBDE-30AB92B243FE}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B317EE0E-6F4B-48FA-8DB9-1B21E52D6EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="44092" windowHeight="24292" xr2:uid="{B86492C5-8FE4-4237-A3C4-CEFE931CA8D1}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13996" xr2:uid="{B86492C5-8FE4-4237-A3C4-CEFE931CA8D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Pricer" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
+  <calcPr calcId="191029" calcMode="manual" calcCompleted="0" calcOnSave="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -220,10 +215,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.00;0.00;"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="0%;\%;"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.00;0.00;"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="167" formatCode="0%;\%;"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -571,7 +566,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
@@ -590,7 +585,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3"/>
@@ -616,7 +611,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="2" applyBorder="1"/>
@@ -624,29 +619,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="11" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="3" fillId="3" borderId="15" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -656,16 +642,7 @@
     <xf numFmtId="9" fontId="3" fillId="3" borderId="6" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="3" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="2" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="10" fillId="6" borderId="4" xfId="7" applyNumberFormat="1" applyBorder="1"/>
@@ -679,6 +656,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="10" fillId="6" borderId="17" xfId="7" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Bad" xfId="6" builtinId="27"/>
@@ -1001,36 +996,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{311DAF8B-FD97-4102-B095-760DF1A411B5}">
   <dimension ref="B1:V118"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="16" max="16" width="11.07421875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="30.07421875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.06640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45"/>
-    <row r="2" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C2" s="7" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F2" s="45" t="s">
+      <c r="F2" s="39" t="s">
         <v>59</v>
       </c>
-      <c r="J2" s="47" t="s">
+      <c r="J2" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="46" t="str">
+      <c r="K2" s="40" t="str">
         <f ca="1">_xll.xPutDLM(OFFSET(C9,0,0,$K$8,1),OFFSET(D9,0,0,$K$8,1),OFFSET(E9,0,0,$K$8,1),OFFSET(F9,0,0,$K$8,1),E52,OFFSET(H53,0,0,$K$8,1),OFFSET(C40,0,0,$K$37,1),OFFSET(D40,0,0,$K$37,$K$8),OFFSET(D23,0,0,$K$8,$K$8),K34,"dlm")</f>
         <v>dlm</v>
       </c>
-      <c r="O2" s="32" t="s">
+      <c r="O2" s="43" t="s">
         <v>54</v>
       </c>
-      <c r="P2" s="33"/>
-      <c r="Q2" s="33"/>
-      <c r="R2" s="34"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="45"/>
       <c r="T2" s="15" t="s">
         <v>60</v>
       </c>
@@ -1039,17 +1034,17 @@
         <v>autocall strike 70 KO 100 CPN 32 6 periods of 1m</v>
       </c>
     </row>
-    <row r="3" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="J3" s="47" t="s">
+      <c r="J3" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="K3" s="46" t="str">
+      <c r="K3" s="40" t="str">
         <f ca="1">_xll.xPutAutocall(OFFSET(C9,0,0,$K$8,1),OFFSET(D9,0,0,$K$8,1),U4,U5,U6,U7,U8,U9,"autocall")</f>
         <v>autocall</v>
       </c>
@@ -1060,7 +1055,7 @@
       <c r="Q3" s="22"/>
       <c r="R3" s="23"/>
     </row>
-    <row r="4" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.45">
       <c r="O4" s="21"/>
       <c r="P4" s="22"/>
       <c r="Q4" s="22"/>
@@ -1075,7 +1070,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
         <v>2</v>
       </c>
@@ -1098,7 +1093,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
         <v>3</v>
       </c>
@@ -1121,7 +1116,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="O7" s="24" t="s">
         <v>48</v>
       </c>
@@ -1131,14 +1126,14 @@
       <c r="T7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="U7" s="35">
+      <c r="U7" s="32">
         <v>0.7</v>
       </c>
       <c r="V7" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1165,21 +1160,21 @@
       <c r="T8" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="U8" s="37">
+      <c r="U8" s="34">
         <v>0.32408695869419402</v>
       </c>
       <c r="V8" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.45">
       <c r="B9" s="5">
         <v>1</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="41">
+      <c r="D9" s="35">
         <v>31.55</v>
       </c>
       <c r="E9" s="3">
@@ -1197,14 +1192,14 @@
       <c r="T9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="U9" s="36">
+      <c r="U9" s="33">
         <v>0.01</v>
       </c>
       <c r="V9" s="8" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.45">
       <c r="B10" s="5">
         <f>IF(LEN(C10)&gt;0,B9+1,"")</f>
         <v>2</v>
@@ -1212,7 +1207,7 @@
       <c r="C10" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="41">
+      <c r="D10" s="35">
         <v>42</v>
       </c>
       <c r="E10" s="3">
@@ -1228,7 +1223,7 @@
       <c r="Q10" s="22"/>
       <c r="R10" s="23"/>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.45">
       <c r="B11" s="5">
         <f t="shared" ref="B11:B18" si="0">IF(LEN(C11)&gt;0,B10+1,"")</f>
         <v>3</v>
@@ -1236,7 +1231,7 @@
       <c r="C11" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="41">
+      <c r="D11" s="35">
         <v>20</v>
       </c>
       <c r="E11" s="9">
@@ -1264,13 +1259,13 @@
         <v>100000</v>
       </c>
     </row>
-    <row r="12" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C12" s="12"/>
-      <c r="D12" s="41"/>
+      <c r="D12" s="35"/>
       <c r="E12" s="9"/>
       <c r="F12" s="4"/>
       <c r="I12" s="8" t="s">
@@ -1289,49 +1284,49 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B13" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C13" s="12"/>
-      <c r="D13" s="41"/>
+      <c r="D13" s="35"/>
       <c r="E13" s="9"/>
       <c r="F13" s="4"/>
     </row>
-    <row r="14" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B14" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C14" s="12"/>
-      <c r="D14" s="41"/>
+      <c r="D14" s="35"/>
       <c r="E14" s="9"/>
       <c r="F14" s="4"/>
-      <c r="H14" s="32" t="s">
+      <c r="H14" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="34"/>
-    </row>
-    <row r="15" spans="2:22" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="I14" s="44"/>
+      <c r="J14" s="44"/>
+      <c r="K14" s="44"/>
+      <c r="L14" s="45"/>
+    </row>
+    <row r="15" spans="2:22" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C15" s="12"/>
-      <c r="D15" s="41"/>
+      <c r="D15" s="35"/>
       <c r="E15" s="9"/>
       <c r="F15" s="4"/>
-      <c r="H15" s="38" t="s">
+      <c r="H15" s="46" t="s">
         <v>56</v>
       </c>
-      <c r="I15" s="39"/>
-      <c r="J15" s="39"/>
-      <c r="K15" s="39"/>
-      <c r="L15" s="40"/>
+      <c r="I15" s="47"/>
+      <c r="J15" s="47"/>
+      <c r="K15" s="47"/>
+      <c r="L15" s="48"/>
       <c r="O15" s="17" t="s">
         <v>33</v>
       </c>
@@ -1339,48 +1334,48 @@
         <f t="array" aca="1" ref="Q15:R15" ca="1">_xll.xValue(K2,K3,TRUE,,,U11,U12)</f>
         <v>autocall strike 70 KO 100 CPN 32 6 periods of 1m</v>
       </c>
-      <c r="R15" s="44">
-        <f ca="1"/>
-        <v>0.97999999999776122</v>
+      <c r="R15" s="38">
+        <f ca="1"/>
+        <v>0.97999999999776133</v>
       </c>
       <c r="S15" s="18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.45">
       <c r="B16" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C16" s="12"/>
-      <c r="D16" s="41"/>
+      <c r="D16" s="35"/>
       <c r="E16" s="9"/>
       <c r="F16" s="4"/>
     </row>
-    <row r="17" spans="2:19" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:19" x14ac:dyDescent="0.45">
       <c r="B17" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C17" s="12"/>
-      <c r="D17" s="41"/>
+      <c r="D17" s="35"/>
       <c r="E17" s="9"/>
       <c r="F17" s="4"/>
       <c r="O17" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B18" s="5" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="C18" s="13"/>
-      <c r="D18" s="41"/>
+      <c r="D18" s="35"/>
       <c r="E18" s="9"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" spans="2:19" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="O19" s="17" t="s">
         <v>38</v>
       </c>
@@ -1388,15 +1383,15 @@
         <f t="array" aca="1" ref="Q19:R118" ca="1">_xll.xAADrisk(K2,K3,U2,TRUE,,,U11,U12)</f>
         <v>value</v>
       </c>
-      <c r="R19" s="44">
-        <f ca="1"/>
-        <v>0.97999999999776122</v>
+      <c r="R19" s="38">
+        <f ca="1"/>
+        <v>0.97999999999776133</v>
       </c>
       <c r="S19" s="18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="2:19" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C20" s="8" t="s">
         <v>8</v>
       </c>
@@ -1404,25 +1399,25 @@
         <f ca="1"/>
         <v>disc rate</v>
       </c>
-      <c r="R20" s="48">
-        <f ca="1"/>
-        <v>-0.14378218975556961</v>
+      <c r="R20" s="42">
+        <f ca="1"/>
+        <v>-0.1437821897555695</v>
       </c>
       <c r="S20" s="18" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="2:19" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:19" x14ac:dyDescent="0.45">
       <c r="Q21" s="5" t="str">
         <f ca="1"/>
         <v>spot uber</v>
       </c>
-      <c r="R21" s="42">
-        <f ca="1"/>
-        <v>1.6811137718893772E-4</v>
-      </c>
-    </row>
-    <row r="22" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R21" s="36">
+        <f ca="1"/>
+        <v>1.6811137718893645E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C22" s="6"/>
       <c r="D22" s="6" t="str">
         <f t="array" ref="D22:M22">TRANSPOSE(C23:C32)</f>
@@ -1459,12 +1454,12 @@
         <f ca="1"/>
         <v>spot lyft</v>
       </c>
-      <c r="R22" s="42">
-        <f ca="1"/>
-        <v>8.3920819726307364E-4</v>
-      </c>
-    </row>
-    <row r="23" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R22" s="36">
+        <f ca="1"/>
+        <v>8.3920819726307743E-4</v>
+      </c>
+    </row>
+    <row r="23" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C23" s="6" t="str">
         <f t="array" ref="C23:C32">IF(LEN(C9:C18)&gt;0,C9:C18,"")</f>
         <v>uber</v>
@@ -1504,12 +1499,12 @@
         <f ca="1"/>
         <v>spot luckin</v>
       </c>
-      <c r="R23" s="42">
-        <f ca="1"/>
-        <v>5.3909429623618344E-3</v>
-      </c>
-    </row>
-    <row r="24" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R23" s="36">
+        <f ca="1"/>
+        <v>5.3909429623618336E-3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C24" s="6" t="str">
         <v>lyft</v>
       </c>
@@ -1548,12 +1543,12 @@
         <f ca="1"/>
         <v>repo spread uber</v>
       </c>
-      <c r="R24" s="42">
-        <f ca="1"/>
-        <v>-1.4698674508598795E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R24" s="36">
+        <f ca="1"/>
+        <v>-1.4698674508598788E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C25" s="6" t="str">
         <v>luckin</v>
       </c>
@@ -1592,12 +1587,12 @@
         <f ca="1"/>
         <v>repo spread lyft</v>
       </c>
-      <c r="R25" s="42">
-        <f ca="1"/>
-        <v>-6.6959506590848025E-2</v>
-      </c>
-    </row>
-    <row r="26" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R25" s="36">
+        <f ca="1"/>
+        <v>-6.6959506590847997E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C26" s="6" t="str">
         <v/>
       </c>
@@ -1630,12 +1625,12 @@
         <f ca="1"/>
         <v>repo spread luckin</v>
       </c>
-      <c r="R26" s="42">
-        <f ca="1"/>
-        <v>-6.6339138885223553E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R26" s="36">
+        <f ca="1"/>
+        <v>-6.6339138885223539E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C27" s="6" t="str">
         <v/>
       </c>
@@ -1666,12 +1661,12 @@
         <f ca="1"/>
         <v>div uber 0.25</v>
       </c>
-      <c r="R27" s="42">
-        <f ca="1"/>
-        <v>-3.3784336373654737E-2</v>
-      </c>
-    </row>
-    <row r="28" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R27" s="36">
+        <f ca="1"/>
+        <v>-3.378433637365473E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C28" s="6" t="str">
         <v/>
       </c>
@@ -1700,12 +1695,12 @@
         <f ca="1"/>
         <v>div lyft 0.25</v>
       </c>
-      <c r="R28" s="42">
-        <f ca="1"/>
-        <v>-0.11079783359950626</v>
-      </c>
-    </row>
-    <row r="29" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R28" s="36">
+        <f ca="1"/>
+        <v>-0.11079783359950625</v>
+      </c>
+    </row>
+    <row r="29" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C29" s="6" t="str">
         <v/>
       </c>
@@ -1732,12 +1727,12 @@
         <f ca="1"/>
         <v>div luckin 0.25</v>
       </c>
-      <c r="R29" s="42">
-        <f ca="1"/>
-        <v>-0.12948155244360332</v>
-      </c>
-    </row>
-    <row r="30" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R29" s="36">
+        <f ca="1"/>
+        <v>-0.12948155244360329</v>
+      </c>
+    </row>
+    <row r="30" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C30" s="6" t="str">
         <v/>
       </c>
@@ -1762,12 +1757,12 @@
         <f ca="1"/>
         <v>div uber 0.50</v>
       </c>
-      <c r="R30" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R30" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C31" s="6" t="str">
         <v/>
       </c>
@@ -1790,12 +1785,12 @@
         <f ca="1"/>
         <v>div lyft 0.50</v>
       </c>
-      <c r="R31" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="2:19" x14ac:dyDescent="0.4">
+      <c r="R31" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:19" x14ac:dyDescent="0.45">
       <c r="C32" s="6" t="str">
         <v/>
       </c>
@@ -1815,22 +1810,22 @@
         <f ca="1"/>
         <v>div luckin 0.50</v>
       </c>
-      <c r="R32" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R32" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="2:18" x14ac:dyDescent="0.45">
       <c r="Q33" s="5" t="str">
         <f ca="1"/>
         <v>div uber 0.75</v>
       </c>
-      <c r="R33" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R33" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:18" x14ac:dyDescent="0.45">
       <c r="C34" s="8" t="s">
         <v>19</v>
       </c>
@@ -1844,22 +1839,22 @@
         <f ca="1"/>
         <v>div lyft 0.75</v>
       </c>
-      <c r="R34" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R34" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="2:18" x14ac:dyDescent="0.45">
       <c r="Q35" s="5" t="str">
         <f ca="1"/>
         <v>div luckin 0.75</v>
       </c>
-      <c r="R35" s="42">
-        <f ca="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R35" s="36">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:18" x14ac:dyDescent="0.45">
       <c r="C36" s="8" t="s">
         <v>37</v>
       </c>
@@ -1867,12 +1862,12 @@
         <f ca="1"/>
         <v>ATM uber</v>
       </c>
-      <c r="R36" s="42">
-        <f ca="1"/>
-        <v>-4.7866615287150846E-2</v>
-      </c>
-    </row>
-    <row r="37" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R36" s="36">
+        <f ca="1"/>
+        <v>-4.7866615287150818E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="2:18" x14ac:dyDescent="0.45">
       <c r="C37" s="8" t="s">
         <v>36</v>
       </c>
@@ -1887,23 +1882,23 @@
         <f ca="1"/>
         <v>ATM lyft</v>
       </c>
-      <c r="R37" s="42">
-        <f ca="1"/>
-        <v>-0.15670370202633022</v>
-      </c>
-    </row>
-    <row r="38" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R37" s="36">
+        <f ca="1"/>
+        <v>-0.15670370202632988</v>
+      </c>
+    </row>
+    <row r="38" spans="2:18" x14ac:dyDescent="0.45">
       <c r="K38" s="20"/>
       <c r="Q38" s="5" t="str">
         <f ca="1"/>
         <v>ATM luckin</v>
       </c>
-      <c r="R38" s="42">
-        <f ca="1"/>
-        <v>-0.15259801016064761</v>
-      </c>
-    </row>
-    <row r="39" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="R38" s="36">
+        <f ca="1"/>
+        <v>-0.1525980101606477</v>
+      </c>
+    </row>
+    <row r="39" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C39" s="1" t="s">
         <v>11</v>
       </c>
@@ -1942,12 +1937,12 @@
         <f ca="1"/>
         <v>skew uber</v>
       </c>
-      <c r="R39" s="42">
-        <f ca="1"/>
-        <v>2.1439903798762844E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R39" s="36">
+        <f ca="1"/>
+        <v>2.1439903798762944E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B40" s="5">
         <v>1</v>
       </c>
@@ -1972,12 +1967,12 @@
         <f ca="1"/>
         <v>skew lyft</v>
       </c>
-      <c r="R40" s="42">
-        <f ca="1"/>
-        <v>6.7053341249287898E-2</v>
-      </c>
-    </row>
-    <row r="41" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R40" s="36">
+        <f ca="1"/>
+        <v>6.7053341249288176E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B41" s="5">
         <f>IF(LEN(C41)&gt;0,B40+1,"")</f>
         <v>2</v>
@@ -2003,12 +1998,12 @@
         <f ca="1"/>
         <v>skew luckin</v>
       </c>
-      <c r="R41" s="42">
-        <f ca="1"/>
-        <v>7.9247786640885942E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R41" s="36">
+        <f ca="1"/>
+        <v>7.9247786640885026E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B42" s="5">
         <f t="shared" ref="B42:B49" si="1">IF(LEN(C42)&gt;0,B41+1,"")</f>
         <v>3</v>
@@ -2034,12 +2029,12 @@
         <f ca="1"/>
         <v>correl lyft uber</v>
       </c>
-      <c r="R42" s="42">
-        <f ca="1"/>
-        <v>7.1265585287710858E-3</v>
-      </c>
-    </row>
-    <row r="43" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R42" s="36">
+        <f ca="1"/>
+        <v>7.1265585287710971E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B43" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2059,12 +2054,12 @@
         <f ca="1"/>
         <v>correl luckin uber</v>
       </c>
-      <c r="R43" s="42">
-        <f ca="1"/>
-        <v>3.894576595381857E-3</v>
-      </c>
-    </row>
-    <row r="44" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R43" s="36">
+        <f ca="1"/>
+        <v>3.8945765953818517E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B44" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2084,12 +2079,12 @@
         <f ca="1"/>
         <v>correl luckin lyft</v>
       </c>
-      <c r="R44" s="42">
-        <f ca="1"/>
-        <v>1.4406372025372786E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R44" s="36">
+        <f ca="1"/>
+        <v>1.4406372025372784E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B45" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2109,12 +2104,12 @@
         <f ca="1"/>
         <v>lambda</v>
       </c>
-      <c r="R45" s="42">
-        <f ca="1"/>
-        <v>1.9931508790879432E-2</v>
-      </c>
-    </row>
-    <row r="46" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R45" s="36">
+        <f ca="1"/>
+        <v>1.9931508790879428E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B46" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2134,12 +2129,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R46" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="47" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R46" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="47" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B47" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2159,12 +2154,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R47" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="48" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R47" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="48" spans="2:18" x14ac:dyDescent="0.45">
       <c r="B48" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2184,12 +2179,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R48" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="49" spans="2:18" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="R48" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="49" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B49" s="5" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2209,22 +2204,22 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R49" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="50" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R49" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="50" spans="2:18" x14ac:dyDescent="0.45">
       <c r="Q50" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R50" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R50" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="51" spans="2:18" x14ac:dyDescent="0.45">
       <c r="C51" s="8" t="s">
         <v>52</v>
       </c>
@@ -2235,12 +2230,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R51" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R51" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="52" spans="2:18" x14ac:dyDescent="0.45">
       <c r="C52" s="5" t="s">
         <v>13</v>
       </c>
@@ -2259,12 +2254,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R52" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R52" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="53" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G53" s="1" t="str">
         <f t="array" ref="G53:G62">C23:C32</f>
         <v>uber</v>
@@ -2276,12 +2271,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R53" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R53" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="54" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G54" s="1" t="str">
         <v>lyft</v>
       </c>
@@ -2292,12 +2287,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R54" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="55" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R54" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="55" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G55" s="1" t="str">
         <v>luckin</v>
       </c>
@@ -2308,12 +2303,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R55" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="56" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R55" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="56" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G56" s="1" t="str">
         <v/>
       </c>
@@ -2322,12 +2317,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R56" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="57" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R56" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="57" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G57" s="1" t="str">
         <v/>
       </c>
@@ -2336,12 +2331,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R57" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="58" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R57" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="58" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G58" s="1" t="str">
         <v/>
       </c>
@@ -2350,12 +2345,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R58" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="59" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R58" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="59" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G59" s="1" t="str">
         <v/>
       </c>
@@ -2364,12 +2359,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R59" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="60" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R59" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="60" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G60" s="1" t="str">
         <v/>
       </c>
@@ -2378,12 +2373,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R60" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="61" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R60" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="61" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G61" s="1" t="str">
         <v/>
       </c>
@@ -2392,12 +2387,12 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R61" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="62" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R61" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="62" spans="2:18" x14ac:dyDescent="0.45">
       <c r="G62" s="1" t="str">
         <v/>
       </c>
@@ -2406,567 +2401,567 @@
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R62" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="63" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R62" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="63" spans="2:18" x14ac:dyDescent="0.45">
       <c r="Q63" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R63" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="64" spans="2:18" x14ac:dyDescent="0.4">
+      <c r="R63" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="64" spans="2:18" x14ac:dyDescent="0.45">
       <c r="Q64" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R64" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="65" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R64" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="65" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q65" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R65" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="66" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R65" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="66" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q66" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R66" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="67" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R66" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="67" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q67" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R67" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="68" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R67" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="68" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q68" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R68" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="69" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R68" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="69" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q69" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R69" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="70" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R69" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="70" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q70" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R70" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="71" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R70" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="71" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q71" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R71" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="72" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R71" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="72" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q72" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R72" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="73" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R72" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="73" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q73" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R73" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="74" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R73" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="74" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q74" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R74" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="75" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R74" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="75" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q75" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R75" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="76" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R75" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="76" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q76" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R76" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="77" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R76" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="77" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q77" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R77" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="78" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R77" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="78" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q78" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R78" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="79" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R78" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="79" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q79" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R79" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="80" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R79" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="80" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q80" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R80" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="81" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R80" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="81" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q81" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R81" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="82" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R81" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="82" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q82" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R82" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="83" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R82" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="83" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q83" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R83" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="84" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R83" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="84" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q84" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R84" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="85" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R84" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="85" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q85" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R85" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="86" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R85" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="86" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q86" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R86" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="87" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R86" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="87" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q87" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R87" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="88" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R87" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="88" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q88" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R88" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="89" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R88" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="89" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q89" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R89" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="90" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R89" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="90" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q90" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R90" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="91" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R90" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="91" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q91" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R91" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="92" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R91" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="92" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q92" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R92" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="93" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R92" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="93" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q93" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R93" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="94" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R93" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="94" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q94" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R94" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="95" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R94" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="95" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q95" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R95" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="96" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R95" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="96" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q96" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R96" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="97" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R96" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="97" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q97" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R97" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="98" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R97" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="98" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q98" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R98" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="99" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R98" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="99" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q99" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R99" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="100" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R99" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="100" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q100" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R100" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="101" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R100" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="101" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q101" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R101" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="102" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R101" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="102" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q102" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R102" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="103" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R102" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="103" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q103" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R103" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="104" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R103" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="104" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q104" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R104" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="105" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R104" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="105" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q105" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R105" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="106" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R105" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="106" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q106" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R106" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="107" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R106" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="107" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q107" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R107" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="108" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R107" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="108" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q108" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R108" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="109" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R108" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="109" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q109" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R109" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="110" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R109" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="110" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q110" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R110" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="111" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R110" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="111" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q111" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R111" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="112" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R111" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="112" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q112" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R112" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="113" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R112" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="113" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q113" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R113" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="114" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R113" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="114" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q114" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R114" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="115" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R114" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="115" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q115" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R115" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="116" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R115" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="116" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q116" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R116" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="117" spans="17:18" x14ac:dyDescent="0.4">
+      <c r="R116" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="117" spans="17:18" x14ac:dyDescent="0.45">
       <c r="Q117" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R117" s="42" t="e">
-        <f ca="1"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="118" spans="17:18" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="R117" s="36" t="e">
+        <f ca="1"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="118" spans="17:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="Q118" s="5" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>
-      <c r="R118" s="43" t="e">
+      <c r="R118" s="37" t="e">
         <f ca="1"/>
         <v>#N/A</v>
       </c>

</xml_diff>